<commit_message>
Update derived data files and enhance notebook outputs with file paths
- Updated binary files: club_ranges.xlsx, club_selector.xlsx, clutch_score_analysis.xlsx, golf_recommendations.xlsx, round_profiles.xlsx, strokes_gained_summary.xlsx, and Golf Stats.xlsx.
- Modified Golf Analytics.ipynb to include detailed output messages with full file paths for saved Excel files and adjusted execution counts for code cells.
</commit_message>
<xml_diff>
--- a/data/derived/clutch_score_analysis.xlsx
+++ b/data/derived/clutch_score_analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="36">
   <si>
     <t>Golfer</t>
   </si>
@@ -85,6 +85,9 @@
     <t>Black Bear</t>
   </si>
   <si>
+    <t>Bethpage Red</t>
+  </si>
+  <si>
     <t>Willow Creek Hamlet Course</t>
   </si>
   <si>
@@ -104,9 +107,6 @@
   </si>
   <si>
     <t>Bethpage Black</t>
-  </si>
-  <si>
-    <t>Bethpage Red</t>
   </si>
   <si>
     <t>Sebonack Golf Club</t>
@@ -483,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1155,28 +1155,28 @@
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B24" s="2">
-        <v>45453</v>
+        <v>46243</v>
       </c>
       <c r="C24" t="s">
         <v>23</v>
       </c>
       <c r="D24">
-        <v>2.2</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E24">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F24">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="G24">
-        <v>2.556</v>
+        <v>2.478</v>
       </c>
       <c r="H24">
-        <v>0.027</v>
+        <v>-0.055</v>
       </c>
       <c r="I24" t="s">
         <v>35</v>
@@ -1187,25 +1187,25 @@
         <v>10</v>
       </c>
       <c r="B25" s="2">
-        <v>45492</v>
+        <v>45453</v>
       </c>
       <c r="C25" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D25">
-        <v>2.067</v>
+        <v>2.2</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F25">
-        <v>5.2</v>
+        <v>1.6</v>
       </c>
       <c r="G25">
-        <v>5.894</v>
+        <v>2.556</v>
       </c>
       <c r="H25">
-        <v>-0.122</v>
+        <v>0.027</v>
       </c>
       <c r="I25" t="s">
         <v>35</v>
@@ -1216,28 +1216,28 @@
         <v>10</v>
       </c>
       <c r="B26" s="2">
-        <v>45520</v>
+        <v>45492</v>
       </c>
       <c r="C26" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D26">
-        <v>1.4</v>
+        <v>2.067</v>
       </c>
       <c r="E26">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F26">
-        <v>-1.8</v>
+        <v>5.2</v>
       </c>
       <c r="G26">
-        <v>-2.139</v>
+        <v>5.894</v>
       </c>
       <c r="H26">
-        <v>0.046</v>
+        <v>-0.122</v>
       </c>
       <c r="I26" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1245,28 +1245,28 @@
         <v>10</v>
       </c>
       <c r="B27" s="2">
-        <v>45765</v>
+        <v>45520</v>
       </c>
       <c r="C27" t="s">
         <v>25</v>
       </c>
       <c r="D27">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
       <c r="E27">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F27">
-        <v>3.2</v>
+        <v>-1.8</v>
       </c>
       <c r="G27">
-        <v>3.817</v>
+        <v>-2.139</v>
       </c>
       <c r="H27">
-        <v>-0.105</v>
+        <v>0.046</v>
       </c>
       <c r="I27" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1274,28 +1274,28 @@
         <v>10</v>
       </c>
       <c r="B28" s="2">
-        <v>45853</v>
+        <v>45765</v>
       </c>
       <c r="C28" t="s">
         <v>26</v>
       </c>
       <c r="D28">
-        <v>2.067</v>
+        <v>2.4</v>
       </c>
       <c r="E28">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F28">
-        <v>-0.8</v>
+        <v>3.2</v>
       </c>
       <c r="G28">
-        <v>-1.25</v>
+        <v>3.817</v>
       </c>
       <c r="H28">
-        <v>-0.014</v>
+        <v>-0.105</v>
       </c>
       <c r="I28" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1303,28 +1303,28 @@
         <v>10</v>
       </c>
       <c r="B29" s="2">
-        <v>45894</v>
+        <v>45853</v>
       </c>
       <c r="C29" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D29">
-        <v>2.4</v>
+        <v>2.067</v>
       </c>
       <c r="E29">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F29">
-        <v>2.2</v>
+        <v>-0.8</v>
       </c>
       <c r="G29">
-        <v>3.3</v>
+        <v>-1.25</v>
       </c>
       <c r="H29">
-        <v>-0.046</v>
+        <v>-0.014</v>
       </c>
       <c r="I29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1332,25 +1332,25 @@
         <v>10</v>
       </c>
       <c r="B30" s="2">
-        <v>46185</v>
+        <v>45894</v>
       </c>
       <c r="C30" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D30">
-        <v>1.867</v>
+        <v>2.4</v>
       </c>
       <c r="E30">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F30">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="G30">
-        <v>1.517</v>
+        <v>3.3</v>
       </c>
       <c r="H30">
-        <v>-0.095</v>
+        <v>-0.046</v>
       </c>
       <c r="I30" t="s">
         <v>35</v>
@@ -1361,25 +1361,25 @@
         <v>10</v>
       </c>
       <c r="B31" s="2">
-        <v>46204</v>
+        <v>46185</v>
       </c>
       <c r="C31" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D31">
+        <v>1.867</v>
+      </c>
+      <c r="E31">
+        <v>4</v>
+      </c>
+      <c r="F31">
         <v>1.6</v>
       </c>
-      <c r="E31">
-        <v>3</v>
-      </c>
-      <c r="F31">
-        <v>1.8</v>
-      </c>
       <c r="G31">
-        <v>2.356</v>
+        <v>1.517</v>
       </c>
       <c r="H31">
-        <v>-0.008999999999999999</v>
+        <v>-0.095</v>
       </c>
       <c r="I31" t="s">
         <v>35</v>
@@ -1390,25 +1390,25 @@
         <v>10</v>
       </c>
       <c r="B32" s="2">
-        <v>46211</v>
+        <v>46204</v>
       </c>
       <c r="C32" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D32">
-        <v>2.667</v>
+        <v>1.6</v>
       </c>
       <c r="E32">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>1.8</v>
       </c>
       <c r="G32">
-        <v>4.2</v>
+        <v>2.356</v>
       </c>
       <c r="H32">
-        <v>-0.102</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="I32" t="s">
         <v>35</v>
@@ -1416,28 +1416,28 @@
     </row>
     <row r="33" spans="1:9">
       <c r="A33" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B33" s="2">
-        <v>45048</v>
+        <v>46211</v>
       </c>
       <c r="C33" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="D33">
-        <v>1.333</v>
+        <v>2.667</v>
       </c>
       <c r="E33">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F33">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G33">
-        <v>2.183</v>
+        <v>4.2</v>
       </c>
       <c r="H33">
-        <v>0.01</v>
+        <v>-0.102</v>
       </c>
       <c r="I33" t="s">
         <v>35</v>
@@ -1448,25 +1448,25 @@
         <v>11</v>
       </c>
       <c r="B34" s="2">
-        <v>45050</v>
+        <v>45048</v>
       </c>
       <c r="C34" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D34">
-        <v>1.067</v>
+        <v>1.333</v>
       </c>
       <c r="E34">
         <v>2</v>
       </c>
       <c r="F34">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="G34">
-        <v>1.556</v>
+        <v>2.183</v>
       </c>
       <c r="H34">
-        <v>-0.023</v>
+        <v>0.01</v>
       </c>
       <c r="I34" t="s">
         <v>35</v>
@@ -1477,7 +1477,7 @@
         <v>11</v>
       </c>
       <c r="B35" s="2">
-        <v>45053</v>
+        <v>45050</v>
       </c>
       <c r="C35" t="s">
         <v>14</v>
@@ -1486,19 +1486,19 @@
         <v>1.067</v>
       </c>
       <c r="E35">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F35">
-        <v>-1.8</v>
+        <v>1.2</v>
       </c>
       <c r="G35">
-        <v>-2.361</v>
+        <v>1.556</v>
       </c>
       <c r="H35">
-        <v>0.098</v>
+        <v>-0.023</v>
       </c>
       <c r="I35" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -1509,25 +1509,25 @@
         <v>45053</v>
       </c>
       <c r="C36" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D36">
-        <v>1.4</v>
+        <v>1.067</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F36">
-        <v>2.2</v>
+        <v>-1.8</v>
       </c>
       <c r="G36">
-        <v>2.939</v>
+        <v>-2.361</v>
       </c>
       <c r="H36">
-        <v>-0.079</v>
+        <v>0.098</v>
       </c>
       <c r="I36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -1535,25 +1535,25 @@
         <v>11</v>
       </c>
       <c r="B37" s="2">
-        <v>45084</v>
+        <v>45053</v>
       </c>
       <c r="C37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D37">
-        <v>1.133</v>
+        <v>1.4</v>
       </c>
       <c r="E37">
         <v>2</v>
       </c>
       <c r="F37">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="G37">
-        <v>1.733</v>
+        <v>2.939</v>
       </c>
       <c r="H37">
-        <v>-0.055</v>
+        <v>-0.079</v>
       </c>
       <c r="I37" t="s">
         <v>35</v>
@@ -1564,28 +1564,28 @@
         <v>11</v>
       </c>
       <c r="B38" s="2">
-        <v>45137</v>
+        <v>45084</v>
       </c>
       <c r="C38" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D38">
-        <v>0.9330000000000001</v>
+        <v>1.133</v>
       </c>
       <c r="E38">
         <v>2</v>
       </c>
       <c r="F38">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
       <c r="G38">
-        <v>1.283</v>
+        <v>1.733</v>
       </c>
       <c r="H38">
-        <v>-0.006</v>
+        <v>-0.055</v>
       </c>
       <c r="I38" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -1593,28 +1593,28 @@
         <v>11</v>
       </c>
       <c r="B39" s="2">
-        <v>45143</v>
+        <v>45137</v>
       </c>
       <c r="C39" t="s">
         <v>13</v>
       </c>
       <c r="D39">
-        <v>1.067</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F39">
-        <v>2.2</v>
+        <v>0.8</v>
       </c>
       <c r="G39">
-        <v>2.65</v>
+        <v>1.283</v>
       </c>
       <c r="H39">
-        <v>-0.08400000000000001</v>
+        <v>-0.006</v>
       </c>
       <c r="I39" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -1622,28 +1622,28 @@
         <v>11</v>
       </c>
       <c r="B40" s="2">
-        <v>45144</v>
+        <v>45143</v>
       </c>
       <c r="C40" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="D40">
-        <v>1.6</v>
+        <v>1.067</v>
       </c>
       <c r="E40">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F40">
-        <v>0.8</v>
+        <v>2.2</v>
       </c>
       <c r="G40">
-        <v>1.433</v>
+        <v>2.65</v>
       </c>
       <c r="H40">
-        <v>-0.06</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="I40" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -1651,28 +1651,28 @@
         <v>11</v>
       </c>
       <c r="B41" s="2">
-        <v>45156</v>
+        <v>45144</v>
       </c>
       <c r="C41" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D41">
-        <v>1.267</v>
+        <v>1.6</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F41">
-        <v>2.8</v>
+        <v>0.8</v>
       </c>
       <c r="G41">
-        <v>3.972</v>
+        <v>1.433</v>
       </c>
       <c r="H41">
-        <v>-0.062</v>
+        <v>-0.06</v>
       </c>
       <c r="I41" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -1680,28 +1680,28 @@
         <v>11</v>
       </c>
       <c r="B42" s="2">
-        <v>45172</v>
+        <v>45156</v>
       </c>
       <c r="C42" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D42">
-        <v>0.8</v>
+        <v>1.267</v>
       </c>
       <c r="E42">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F42">
-        <v>-1.6</v>
+        <v>2.8</v>
       </c>
       <c r="G42">
-        <v>-2.111</v>
+        <v>3.972</v>
       </c>
       <c r="H42">
-        <v>-0.014</v>
+        <v>-0.062</v>
       </c>
       <c r="I42" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -1709,28 +1709,28 @@
         <v>11</v>
       </c>
       <c r="B43" s="2">
-        <v>45434</v>
+        <v>45172</v>
       </c>
       <c r="C43" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D43">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E43">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F43">
-        <v>0</v>
+        <v>-1.6</v>
       </c>
       <c r="G43">
-        <v>0.161</v>
+        <v>-2.111</v>
       </c>
       <c r="H43">
-        <v>-0.08500000000000001</v>
+        <v>-0.014</v>
       </c>
       <c r="I43" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -1738,28 +1738,28 @@
         <v>11</v>
       </c>
       <c r="B44" s="2">
-        <v>45440</v>
+        <v>45434</v>
       </c>
       <c r="C44" t="s">
         <v>13</v>
       </c>
       <c r="D44">
-        <v>1.067</v>
+        <v>1</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F44">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="G44">
-        <v>2.939</v>
+        <v>0.161</v>
       </c>
       <c r="H44">
-        <v>-0.04</v>
+        <v>-0.08500000000000001</v>
       </c>
       <c r="I44" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -1767,25 +1767,25 @@
         <v>11</v>
       </c>
       <c r="B45" s="2">
-        <v>45443</v>
+        <v>45440</v>
       </c>
       <c r="C45" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D45">
-        <v>1.133</v>
+        <v>1.067</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F45">
-        <v>3.4</v>
+        <v>2.2</v>
       </c>
       <c r="G45">
-        <v>4.128</v>
+        <v>2.939</v>
       </c>
       <c r="H45">
-        <v>-0.09</v>
+        <v>-0.04</v>
       </c>
       <c r="I45" t="s">
         <v>35</v>
@@ -1796,28 +1796,28 @@
         <v>11</v>
       </c>
       <c r="B46" s="2">
-        <v>45453</v>
+        <v>45443</v>
       </c>
       <c r="C46" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D46">
-        <v>1.333</v>
+        <v>1.133</v>
       </c>
       <c r="E46">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F46">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="G46">
-        <v>0.239</v>
+        <v>4.128</v>
       </c>
       <c r="H46">
-        <v>-0.025</v>
+        <v>-0.09</v>
       </c>
       <c r="I46" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -1825,28 +1825,28 @@
         <v>11</v>
       </c>
       <c r="B47" s="2">
-        <v>45465</v>
+        <v>45453</v>
       </c>
       <c r="C47" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D47">
-        <v>1.4</v>
+        <v>1.333</v>
       </c>
       <c r="E47">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F47">
-        <v>-1.8</v>
+        <v>0</v>
       </c>
       <c r="G47">
-        <v>-2.367</v>
+        <v>0.239</v>
       </c>
       <c r="H47">
-        <v>0.022</v>
+        <v>-0.025</v>
       </c>
       <c r="I47" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -1854,28 +1854,28 @@
         <v>11</v>
       </c>
       <c r="B48" s="2">
-        <v>45466</v>
+        <v>45465</v>
       </c>
       <c r="C48" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="D48">
-        <v>0.667</v>
+        <v>1.4</v>
       </c>
       <c r="E48">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F48">
-        <v>1</v>
+        <v>-1.8</v>
       </c>
       <c r="G48">
-        <v>1.383</v>
+        <v>-2.367</v>
       </c>
       <c r="H48">
-        <v>-0.011</v>
+        <v>0.022</v>
       </c>
       <c r="I48" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -1883,28 +1883,28 @@
         <v>11</v>
       </c>
       <c r="B49" s="2">
-        <v>45467</v>
+        <v>45466</v>
       </c>
       <c r="C49" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D49">
-        <v>0.533</v>
+        <v>0.667</v>
       </c>
       <c r="E49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F49">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="G49">
-        <v>2.033</v>
+        <v>1.383</v>
       </c>
       <c r="H49">
-        <v>-0.07000000000000001</v>
+        <v>-0.011</v>
       </c>
       <c r="I49" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -1912,28 +1912,28 @@
         <v>11</v>
       </c>
       <c r="B50" s="2">
-        <v>45475</v>
+        <v>45467</v>
       </c>
       <c r="C50" t="s">
         <v>12</v>
       </c>
       <c r="D50">
-        <v>0.2</v>
+        <v>0.533</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F50">
-        <v>-1.4</v>
+        <v>1.6</v>
       </c>
       <c r="G50">
-        <v>-1.517</v>
+        <v>2.033</v>
       </c>
       <c r="H50">
-        <v>0.024</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="I50" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -1941,28 +1941,28 @@
         <v>11</v>
       </c>
       <c r="B51" s="2">
-        <v>45480</v>
+        <v>45475</v>
       </c>
       <c r="C51" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="D51">
-        <v>0.667</v>
+        <v>0.2</v>
       </c>
       <c r="E51">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F51">
-        <v>2</v>
+        <v>-1.4</v>
       </c>
       <c r="G51">
-        <v>2.494</v>
+        <v>-1.517</v>
       </c>
       <c r="H51">
-        <v>-0.039</v>
+        <v>0.024</v>
       </c>
       <c r="I51" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -1970,28 +1970,28 @@
         <v>11</v>
       </c>
       <c r="B52" s="2">
-        <v>45487</v>
+        <v>45480</v>
       </c>
       <c r="C52" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D52">
-        <v>0.4</v>
+        <v>0.667</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F52">
-        <v>0.2</v>
+        <v>2</v>
       </c>
       <c r="G52">
-        <v>-0.017</v>
+        <v>2.494</v>
       </c>
       <c r="H52">
-        <v>0.008999999999999999</v>
+        <v>-0.039</v>
       </c>
       <c r="I52" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -1999,28 +1999,28 @@
         <v>11</v>
       </c>
       <c r="B53" s="2">
-        <v>45492</v>
+        <v>45487</v>
       </c>
       <c r="C53" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D53">
-        <v>0.667</v>
+        <v>0.4</v>
       </c>
       <c r="E53">
         <v>1</v>
       </c>
       <c r="F53">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="G53">
-        <v>1.35</v>
+        <v>-0.017</v>
       </c>
       <c r="H53">
-        <v>-0.018</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="I53" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -2028,28 +2028,28 @@
         <v>11</v>
       </c>
       <c r="B54" s="2">
-        <v>45496</v>
+        <v>45492</v>
       </c>
       <c r="C54" t="s">
         <v>16</v>
       </c>
       <c r="D54">
-        <v>0.467</v>
+        <v>0.667</v>
       </c>
       <c r="E54">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F54">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="G54">
-        <v>1.783</v>
+        <v>1.35</v>
       </c>
       <c r="H54">
-        <v>-0.011</v>
+        <v>-0.018</v>
       </c>
       <c r="I54" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -2057,28 +2057,28 @@
         <v>11</v>
       </c>
       <c r="B55" s="2">
-        <v>45502</v>
+        <v>45496</v>
       </c>
       <c r="C55" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D55">
-        <v>0.533</v>
+        <v>0.467</v>
       </c>
       <c r="E55">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F55">
-        <v>-2.4</v>
+        <v>1.4</v>
       </c>
       <c r="G55">
-        <v>-3.428</v>
+        <v>1.783</v>
       </c>
       <c r="H55">
-        <v>0.054</v>
+        <v>-0.011</v>
       </c>
       <c r="I55" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -2086,28 +2086,28 @@
         <v>11</v>
       </c>
       <c r="B56" s="2">
-        <v>45514</v>
+        <v>45502</v>
       </c>
       <c r="C56" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D56">
-        <v>0.867</v>
+        <v>0.533</v>
       </c>
       <c r="E56">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F56">
-        <v>2.6</v>
+        <v>-2.4</v>
       </c>
       <c r="G56">
-        <v>3.278</v>
+        <v>-3.428</v>
       </c>
       <c r="H56">
-        <v>-0.07099999999999999</v>
+        <v>0.054</v>
       </c>
       <c r="I56" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -2115,28 +2115,28 @@
         <v>11</v>
       </c>
       <c r="B57" s="2">
-        <v>45535</v>
+        <v>45514</v>
       </c>
       <c r="C57" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D57">
-        <v>0.9330000000000001</v>
+        <v>0.867</v>
       </c>
       <c r="E57">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F57">
-        <v>0.8</v>
+        <v>2.6</v>
       </c>
       <c r="G57">
-        <v>1.011</v>
+        <v>3.278</v>
       </c>
       <c r="H57">
-        <v>-0.05</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="I57" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -2144,28 +2144,28 @@
         <v>11</v>
       </c>
       <c r="B58" s="2">
-        <v>45570</v>
+        <v>45535</v>
       </c>
       <c r="C58" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D58">
-        <v>0.4</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E58">
         <v>2</v>
       </c>
       <c r="F58">
-        <v>-0.8</v>
+        <v>0.8</v>
       </c>
       <c r="G58">
-        <v>-1.1</v>
+        <v>1.011</v>
       </c>
       <c r="H58">
-        <v>0.035</v>
+        <v>-0.05</v>
       </c>
       <c r="I58" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -2173,28 +2173,28 @@
         <v>11</v>
       </c>
       <c r="B59" s="2">
-        <v>45580</v>
+        <v>45570</v>
       </c>
       <c r="C59" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="D59">
-        <v>0.667</v>
+        <v>0.4</v>
       </c>
       <c r="E59">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F59">
-        <v>1</v>
+        <v>-0.8</v>
       </c>
       <c r="G59">
-        <v>1.056</v>
+        <v>-1.1</v>
       </c>
       <c r="H59">
-        <v>-0.013</v>
+        <v>0.035</v>
       </c>
       <c r="I59" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -2202,28 +2202,28 @@
         <v>11</v>
       </c>
       <c r="B60" s="2">
-        <v>45649</v>
+        <v>45580</v>
       </c>
       <c r="C60" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D60">
-        <v>0.9330000000000001</v>
+        <v>0.667</v>
       </c>
       <c r="E60">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F60">
-        <v>-0.2</v>
+        <v>1</v>
       </c>
       <c r="G60">
-        <v>-0.289</v>
+        <v>1.056</v>
       </c>
       <c r="H60">
-        <v>-0.028</v>
+        <v>-0.013</v>
       </c>
       <c r="I60" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -2231,28 +2231,28 @@
         <v>11</v>
       </c>
       <c r="B61" s="2">
-        <v>45653</v>
+        <v>45649</v>
       </c>
       <c r="C61" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D61">
-        <v>0.4</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F61">
-        <v>-0.8</v>
+        <v>-0.2</v>
       </c>
       <c r="G61">
-        <v>-0.844</v>
+        <v>-0.289</v>
       </c>
       <c r="H61">
-        <v>-0.012</v>
+        <v>-0.028</v>
       </c>
       <c r="I61" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -2260,28 +2260,28 @@
         <v>11</v>
       </c>
       <c r="B62" s="2">
-        <v>45655</v>
+        <v>45653</v>
       </c>
       <c r="C62" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D62">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="E62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F62">
-        <v>1.4</v>
+        <v>-0.8</v>
       </c>
       <c r="G62">
-        <v>1.989</v>
+        <v>-0.844</v>
       </c>
       <c r="H62">
-        <v>0.003</v>
+        <v>-0.012</v>
       </c>
       <c r="I62" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -2289,28 +2289,28 @@
         <v>11</v>
       </c>
       <c r="B63" s="2">
-        <v>45735</v>
+        <v>45655</v>
       </c>
       <c r="C63" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D63">
-        <v>0.333</v>
+        <v>0.8</v>
       </c>
       <c r="E63">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F63">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="G63">
-        <v>1.189</v>
+        <v>1.989</v>
       </c>
       <c r="H63">
-        <v>-0.051</v>
+        <v>0.003</v>
       </c>
       <c r="I63" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -2318,25 +2318,25 @@
         <v>11</v>
       </c>
       <c r="B64" s="2">
-        <v>45829</v>
+        <v>45735</v>
       </c>
       <c r="C64" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D64">
-        <v>0.267</v>
+        <v>0.333</v>
       </c>
       <c r="E64">
         <v>0</v>
       </c>
       <c r="F64">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="G64">
-        <v>0.911</v>
+        <v>1.189</v>
       </c>
       <c r="H64">
-        <v>-0.033</v>
+        <v>-0.051</v>
       </c>
       <c r="I64" t="s">
         <v>33</v>
@@ -2347,25 +2347,25 @@
         <v>11</v>
       </c>
       <c r="B65" s="2">
-        <v>45831</v>
+        <v>45829</v>
       </c>
       <c r="C65" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D65">
-        <v>0.4</v>
+        <v>0.267</v>
       </c>
       <c r="E65">
         <v>0</v>
       </c>
       <c r="F65">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="G65">
-        <v>1.483</v>
+        <v>0.911</v>
       </c>
       <c r="H65">
-        <v>-0.068</v>
+        <v>-0.033</v>
       </c>
       <c r="I65" t="s">
         <v>33</v>
@@ -2376,25 +2376,25 @@
         <v>11</v>
       </c>
       <c r="B66" s="2">
-        <v>45844</v>
+        <v>45831</v>
       </c>
       <c r="C66" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D66">
-        <v>0.467</v>
+        <v>0.4</v>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F66">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="G66">
-        <v>0.628</v>
+        <v>1.483</v>
       </c>
       <c r="H66">
-        <v>0.027</v>
+        <v>-0.068</v>
       </c>
       <c r="I66" t="s">
         <v>33</v>
@@ -2405,28 +2405,28 @@
         <v>11</v>
       </c>
       <c r="B67" s="2">
-        <v>45857</v>
+        <v>45844</v>
       </c>
       <c r="C67" t="s">
         <v>14</v>
       </c>
       <c r="D67">
-        <v>0.2</v>
+        <v>0.467</v>
       </c>
       <c r="E67">
         <v>1</v>
       </c>
       <c r="F67">
-        <v>-0.4</v>
+        <v>0.4</v>
       </c>
       <c r="G67">
-        <v>-0.433</v>
+        <v>0.628</v>
       </c>
       <c r="H67">
-        <v>0.002</v>
+        <v>0.027</v>
       </c>
       <c r="I67" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -2434,28 +2434,28 @@
         <v>11</v>
       </c>
       <c r="B68" s="2">
-        <v>45868</v>
+        <v>45857</v>
       </c>
       <c r="C68" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="D68">
-        <v>0.667</v>
+        <v>0.2</v>
       </c>
       <c r="E68">
         <v>1</v>
       </c>
       <c r="F68">
-        <v>1</v>
+        <v>-0.4</v>
       </c>
       <c r="G68">
-        <v>1.439</v>
+        <v>-0.433</v>
       </c>
       <c r="H68">
-        <v>0.018</v>
+        <v>0.002</v>
       </c>
       <c r="I68" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -2463,28 +2463,28 @@
         <v>11</v>
       </c>
       <c r="B69" s="2">
-        <v>45886</v>
+        <v>45868</v>
       </c>
       <c r="C69" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D69">
-        <v>0.6</v>
+        <v>0.667</v>
       </c>
       <c r="E69">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F69">
-        <v>-0.2</v>
+        <v>1</v>
       </c>
       <c r="G69">
-        <v>-0.644</v>
+        <v>1.439</v>
       </c>
       <c r="H69">
-        <v>-0.005</v>
+        <v>0.018</v>
       </c>
       <c r="I69" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -2492,28 +2492,28 @@
         <v>11</v>
       </c>
       <c r="B70" s="2">
-        <v>45892</v>
+        <v>45886</v>
       </c>
       <c r="C70" t="s">
         <v>20</v>
       </c>
       <c r="D70">
-        <v>0.733</v>
+        <v>0.6</v>
       </c>
       <c r="E70">
         <v>2</v>
       </c>
       <c r="F70">
-        <v>0.2</v>
+        <v>-0.2</v>
       </c>
       <c r="G70">
-        <v>0.361</v>
+        <v>-0.644</v>
       </c>
       <c r="H70">
-        <v>-0.055</v>
+        <v>-0.005</v>
       </c>
       <c r="I70" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -2521,28 +2521,28 @@
         <v>11</v>
       </c>
       <c r="B71" s="2">
-        <v>45894</v>
+        <v>45892</v>
       </c>
       <c r="C71" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D71">
-        <v>1.2</v>
+        <v>0.733</v>
       </c>
       <c r="E71">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F71">
-        <v>-2.4</v>
+        <v>0.2</v>
       </c>
       <c r="G71">
-        <v>-2.606</v>
+        <v>0.361</v>
       </c>
       <c r="H71">
-        <v>0.068</v>
+        <v>-0.055</v>
       </c>
       <c r="I71" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -2550,25 +2550,25 @@
         <v>11</v>
       </c>
       <c r="B72" s="2">
-        <v>45897</v>
+        <v>45894</v>
       </c>
       <c r="C72" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D72">
-        <v>0.867</v>
+        <v>1.2</v>
       </c>
       <c r="E72">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F72">
-        <v>-1.4</v>
+        <v>-2.4</v>
       </c>
       <c r="G72">
-        <v>-1.789</v>
+        <v>-2.606</v>
       </c>
       <c r="H72">
-        <v>0.001</v>
+        <v>0.068</v>
       </c>
       <c r="I72" t="s">
         <v>34</v>
@@ -2579,25 +2579,25 @@
         <v>11</v>
       </c>
       <c r="B73" s="2">
-        <v>45941</v>
+        <v>45897</v>
       </c>
       <c r="C73" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D73">
-        <v>0.9330000000000001</v>
+        <v>0.867</v>
       </c>
       <c r="E73">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F73">
-        <v>-2.2</v>
+        <v>-1.4</v>
       </c>
       <c r="G73">
-        <v>-2.9</v>
+        <v>-1.789</v>
       </c>
       <c r="H73">
-        <v>-0.001</v>
+        <v>0.001</v>
       </c>
       <c r="I73" t="s">
         <v>34</v>
@@ -2608,25 +2608,25 @@
         <v>11</v>
       </c>
       <c r="B74" s="2">
-        <v>46160</v>
+        <v>45941</v>
       </c>
       <c r="C74" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D74">
-        <v>0.467</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E74">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F74">
-        <v>-1.6</v>
+        <v>-2.2</v>
       </c>
       <c r="G74">
-        <v>-1.972</v>
+        <v>-2.9</v>
       </c>
       <c r="H74">
-        <v>0.029</v>
+        <v>-0.001</v>
       </c>
       <c r="I74" t="s">
         <v>34</v>
@@ -2637,28 +2637,28 @@
         <v>11</v>
       </c>
       <c r="B75" s="2">
-        <v>46164</v>
+        <v>46160</v>
       </c>
       <c r="C75" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D75">
-        <v>1</v>
+        <v>0.467</v>
       </c>
       <c r="E75">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F75">
-        <v>1</v>
+        <v>-1.6</v>
       </c>
       <c r="G75">
-        <v>1.417</v>
+        <v>-1.972</v>
       </c>
       <c r="H75">
-        <v>0.011</v>
+        <v>0.029</v>
       </c>
       <c r="I75" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -2666,28 +2666,28 @@
         <v>11</v>
       </c>
       <c r="B76" s="2">
-        <v>46173</v>
+        <v>46164</v>
       </c>
       <c r="C76" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D76">
-        <v>0.733</v>
+        <v>1</v>
       </c>
       <c r="E76">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F76">
-        <v>-0.8</v>
+        <v>1</v>
       </c>
       <c r="G76">
-        <v>-1.167</v>
+        <v>1.417</v>
       </c>
       <c r="H76">
-        <v>0.023</v>
+        <v>0.011</v>
       </c>
       <c r="I76" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -2695,25 +2695,25 @@
         <v>11</v>
       </c>
       <c r="B77" s="2">
-        <v>46201</v>
+        <v>46173</v>
       </c>
       <c r="C77" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D77">
-        <v>1.067</v>
+        <v>0.733</v>
       </c>
       <c r="E77">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F77">
-        <v>-2.8</v>
+        <v>-0.8</v>
       </c>
       <c r="G77">
-        <v>-3.983</v>
+        <v>-1.167</v>
       </c>
       <c r="H77">
-        <v>0.002</v>
+        <v>0.023</v>
       </c>
       <c r="I77" t="s">
         <v>34</v>
@@ -2724,25 +2724,25 @@
         <v>11</v>
       </c>
       <c r="B78" s="2">
-        <v>46212</v>
+        <v>46201</v>
       </c>
       <c r="C78" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D78">
-        <v>0.4</v>
+        <v>1.067</v>
       </c>
       <c r="E78">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F78">
-        <v>-1.8</v>
+        <v>-2.8</v>
       </c>
       <c r="G78">
-        <v>-2.756</v>
+        <v>-3.983</v>
       </c>
       <c r="H78">
-        <v>0.015</v>
+        <v>0.002</v>
       </c>
       <c r="I78" t="s">
         <v>34</v>
@@ -2753,28 +2753,28 @@
         <v>11</v>
       </c>
       <c r="B79" s="2">
-        <v>46221</v>
+        <v>46212</v>
       </c>
       <c r="C79" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D79">
-        <v>0.867</v>
+        <v>0.4</v>
       </c>
       <c r="E79">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F79">
-        <v>1.6</v>
+        <v>-1.8</v>
       </c>
       <c r="G79">
-        <v>1.85</v>
+        <v>-2.756</v>
       </c>
       <c r="H79">
-        <v>-0.027</v>
+        <v>0.015</v>
       </c>
       <c r="I79" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -2782,10 +2782,10 @@
         <v>11</v>
       </c>
       <c r="B80" s="2">
-        <v>46222</v>
+        <v>46221</v>
       </c>
       <c r="C80" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D80">
         <v>0.867</v>
@@ -2797,13 +2797,71 @@
         <v>1.6</v>
       </c>
       <c r="G80">
-        <v>1.861</v>
+        <v>1.85</v>
       </c>
       <c r="H80">
         <v>-0.027</v>
       </c>
       <c r="I80" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9">
+      <c r="A81" t="s">
+        <v>11</v>
+      </c>
+      <c r="B81" s="2">
+        <v>46222</v>
+      </c>
+      <c r="C81" t="s">
+        <v>22</v>
+      </c>
+      <c r="D81">
+        <v>0.867</v>
+      </c>
+      <c r="E81">
+        <v>1</v>
+      </c>
+      <c r="F81">
+        <v>1.6</v>
+      </c>
+      <c r="G81">
+        <v>1.861</v>
+      </c>
+      <c r="H81">
+        <v>-0.027</v>
+      </c>
+      <c r="I81" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9">
+      <c r="A82" t="s">
+        <v>11</v>
+      </c>
+      <c r="B82" s="2">
+        <v>46243</v>
+      </c>
+      <c r="C82" t="s">
+        <v>23</v>
+      </c>
+      <c r="D82">
+        <v>0.333</v>
+      </c>
+      <c r="E82">
+        <v>0</v>
+      </c>
+      <c r="F82">
+        <v>1</v>
+      </c>
+      <c r="G82">
+        <v>1.089</v>
+      </c>
+      <c r="H82">
+        <v>0.001</v>
+      </c>
+      <c r="I82" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove obsolete mobile visual configurations and update analytics data
- Deleted multiple mobile visual JSON files from the Golf Dashboard 2.0 report, including visuals related to descent angle, club speed, ball speed, and dispersion map.
- Updated the Golf Analytics notebook to reflect changes in round statistics, including adjustments to player performance metrics and baseline means.
- Updated derived Excel files to ensure consistency with the latest data inputs and calculations.
</commit_message>
<xml_diff>
--- a/data/derived/clutch_score_analysis.xlsx
+++ b/data/derived/clutch_score_analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="36">
   <si>
     <t>Golfer</t>
   </si>
@@ -483,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1184,31 +1184,31 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B25" s="2">
-        <v>45453</v>
+        <v>46249</v>
       </c>
       <c r="C25" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="D25">
-        <v>2.2</v>
+        <v>1.133</v>
       </c>
       <c r="E25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F25">
-        <v>1.6</v>
+        <v>-0.6</v>
       </c>
       <c r="G25">
-        <v>2.556</v>
+        <v>-0.878</v>
       </c>
       <c r="H25">
-        <v>0.027</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="I25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1216,25 +1216,25 @@
         <v>10</v>
       </c>
       <c r="B26" s="2">
-        <v>45492</v>
+        <v>45453</v>
       </c>
       <c r="C26" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D26">
-        <v>2.067</v>
+        <v>2.2</v>
       </c>
       <c r="E26">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F26">
-        <v>5.2</v>
+        <v>1.6</v>
       </c>
       <c r="G26">
-        <v>5.894</v>
+        <v>2.556</v>
       </c>
       <c r="H26">
-        <v>-0.122</v>
+        <v>0.027</v>
       </c>
       <c r="I26" t="s">
         <v>35</v>
@@ -1245,28 +1245,28 @@
         <v>10</v>
       </c>
       <c r="B27" s="2">
-        <v>45520</v>
+        <v>45492</v>
       </c>
       <c r="C27" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="D27">
-        <v>1.4</v>
+        <v>2.067</v>
       </c>
       <c r="E27">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F27">
-        <v>-1.8</v>
+        <v>5.2</v>
       </c>
       <c r="G27">
-        <v>-2.139</v>
+        <v>5.894</v>
       </c>
       <c r="H27">
-        <v>0.046</v>
+        <v>-0.122</v>
       </c>
       <c r="I27" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1274,28 +1274,28 @@
         <v>10</v>
       </c>
       <c r="B28" s="2">
-        <v>45765</v>
+        <v>45520</v>
       </c>
       <c r="C28" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D28">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
       <c r="E28">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F28">
-        <v>3.2</v>
+        <v>-1.8</v>
       </c>
       <c r="G28">
-        <v>3.817</v>
+        <v>-2.139</v>
       </c>
       <c r="H28">
-        <v>-0.105</v>
+        <v>0.046</v>
       </c>
       <c r="I28" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1303,28 +1303,28 @@
         <v>10</v>
       </c>
       <c r="B29" s="2">
-        <v>45853</v>
+        <v>45765</v>
       </c>
       <c r="C29" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D29">
-        <v>2.067</v>
+        <v>2.4</v>
       </c>
       <c r="E29">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F29">
-        <v>-0.8</v>
+        <v>3.2</v>
       </c>
       <c r="G29">
-        <v>-1.25</v>
+        <v>3.817</v>
       </c>
       <c r="H29">
-        <v>-0.014</v>
+        <v>-0.105</v>
       </c>
       <c r="I29" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1332,28 +1332,28 @@
         <v>10</v>
       </c>
       <c r="B30" s="2">
-        <v>45894</v>
+        <v>45853</v>
       </c>
       <c r="C30" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D30">
-        <v>2.4</v>
+        <v>2.067</v>
       </c>
       <c r="E30">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F30">
-        <v>2.2</v>
+        <v>-0.8</v>
       </c>
       <c r="G30">
-        <v>3.3</v>
+        <v>-1.25</v>
       </c>
       <c r="H30">
-        <v>-0.046</v>
+        <v>-0.014</v>
       </c>
       <c r="I30" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1361,25 +1361,25 @@
         <v>10</v>
       </c>
       <c r="B31" s="2">
-        <v>46185</v>
+        <v>45894</v>
       </c>
       <c r="C31" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D31">
-        <v>1.867</v>
+        <v>2.4</v>
       </c>
       <c r="E31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F31">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="G31">
-        <v>1.517</v>
+        <v>3.3</v>
       </c>
       <c r="H31">
-        <v>-0.095</v>
+        <v>-0.046</v>
       </c>
       <c r="I31" t="s">
         <v>35</v>
@@ -1390,25 +1390,25 @@
         <v>10</v>
       </c>
       <c r="B32" s="2">
-        <v>46204</v>
+        <v>46185</v>
       </c>
       <c r="C32" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D32">
+        <v>1.867</v>
+      </c>
+      <c r="E32">
+        <v>4</v>
+      </c>
+      <c r="F32">
         <v>1.6</v>
       </c>
-      <c r="E32">
-        <v>3</v>
-      </c>
-      <c r="F32">
-        <v>1.8</v>
-      </c>
       <c r="G32">
-        <v>2.356</v>
+        <v>1.517</v>
       </c>
       <c r="H32">
-        <v>-0.008999999999999999</v>
+        <v>-0.095</v>
       </c>
       <c r="I32" t="s">
         <v>35</v>
@@ -1419,25 +1419,25 @@
         <v>10</v>
       </c>
       <c r="B33" s="2">
-        <v>46211</v>
+        <v>46204</v>
       </c>
       <c r="C33" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D33">
-        <v>2.667</v>
+        <v>1.6</v>
       </c>
       <c r="E33">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F33">
-        <v>3</v>
+        <v>1.8</v>
       </c>
       <c r="G33">
-        <v>4.2</v>
+        <v>2.356</v>
       </c>
       <c r="H33">
-        <v>-0.102</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="I33" t="s">
         <v>35</v>
@@ -1445,28 +1445,28 @@
     </row>
     <row r="34" spans="1:9">
       <c r="A34" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B34" s="2">
-        <v>45048</v>
+        <v>46211</v>
       </c>
       <c r="C34" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="D34">
-        <v>1.333</v>
+        <v>2.667</v>
       </c>
       <c r="E34">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F34">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G34">
-        <v>2.183</v>
+        <v>4.2</v>
       </c>
       <c r="H34">
-        <v>0.01</v>
+        <v>-0.102</v>
       </c>
       <c r="I34" t="s">
         <v>35</v>
@@ -1477,25 +1477,25 @@
         <v>11</v>
       </c>
       <c r="B35" s="2">
-        <v>45050</v>
+        <v>45048</v>
       </c>
       <c r="C35" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D35">
-        <v>1.067</v>
+        <v>1.333</v>
       </c>
       <c r="E35">
         <v>2</v>
       </c>
       <c r="F35">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="G35">
-        <v>1.556</v>
+        <v>2.183</v>
       </c>
       <c r="H35">
-        <v>-0.023</v>
+        <v>0.01</v>
       </c>
       <c r="I35" t="s">
         <v>35</v>
@@ -1506,7 +1506,7 @@
         <v>11</v>
       </c>
       <c r="B36" s="2">
-        <v>45053</v>
+        <v>45050</v>
       </c>
       <c r="C36" t="s">
         <v>14</v>
@@ -1515,19 +1515,19 @@
         <v>1.067</v>
       </c>
       <c r="E36">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F36">
-        <v>-1.8</v>
+        <v>1.2</v>
       </c>
       <c r="G36">
-        <v>-2.361</v>
+        <v>1.556</v>
       </c>
       <c r="H36">
-        <v>0.098</v>
+        <v>-0.023</v>
       </c>
       <c r="I36" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -1538,25 +1538,25 @@
         <v>45053</v>
       </c>
       <c r="C37" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D37">
-        <v>1.4</v>
+        <v>1.067</v>
       </c>
       <c r="E37">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F37">
-        <v>2.2</v>
+        <v>-1.8</v>
       </c>
       <c r="G37">
-        <v>2.939</v>
+        <v>-2.361</v>
       </c>
       <c r="H37">
-        <v>-0.079</v>
+        <v>0.098</v>
       </c>
       <c r="I37" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -1564,25 +1564,25 @@
         <v>11</v>
       </c>
       <c r="B38" s="2">
-        <v>45084</v>
+        <v>45053</v>
       </c>
       <c r="C38" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D38">
-        <v>1.133</v>
+        <v>1.4</v>
       </c>
       <c r="E38">
         <v>2</v>
       </c>
       <c r="F38">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="G38">
-        <v>1.733</v>
+        <v>2.939</v>
       </c>
       <c r="H38">
-        <v>-0.055</v>
+        <v>-0.079</v>
       </c>
       <c r="I38" t="s">
         <v>35</v>
@@ -1593,28 +1593,28 @@
         <v>11</v>
       </c>
       <c r="B39" s="2">
-        <v>45137</v>
+        <v>45084</v>
       </c>
       <c r="C39" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D39">
-        <v>0.9330000000000001</v>
+        <v>1.133</v>
       </c>
       <c r="E39">
         <v>2</v>
       </c>
       <c r="F39">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
       <c r="G39">
-        <v>1.283</v>
+        <v>1.733</v>
       </c>
       <c r="H39">
-        <v>-0.006</v>
+        <v>-0.055</v>
       </c>
       <c r="I39" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -1622,28 +1622,28 @@
         <v>11</v>
       </c>
       <c r="B40" s="2">
-        <v>45143</v>
+        <v>45137</v>
       </c>
       <c r="C40" t="s">
         <v>13</v>
       </c>
       <c r="D40">
-        <v>1.067</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E40">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F40">
-        <v>2.2</v>
+        <v>0.8</v>
       </c>
       <c r="G40">
-        <v>2.65</v>
+        <v>1.283</v>
       </c>
       <c r="H40">
-        <v>-0.08400000000000001</v>
+        <v>-0.006</v>
       </c>
       <c r="I40" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -1651,28 +1651,28 @@
         <v>11</v>
       </c>
       <c r="B41" s="2">
-        <v>45144</v>
+        <v>45143</v>
       </c>
       <c r="C41" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D41">
-        <v>1.6</v>
+        <v>1.067</v>
       </c>
       <c r="E41">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F41">
-        <v>0.8</v>
+        <v>2.2</v>
       </c>
       <c r="G41">
-        <v>1.433</v>
+        <v>2.65</v>
       </c>
       <c r="H41">
-        <v>-0.06</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="I41" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -1680,28 +1680,28 @@
         <v>11</v>
       </c>
       <c r="B42" s="2">
-        <v>45156</v>
+        <v>45144</v>
       </c>
       <c r="C42" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D42">
-        <v>1.267</v>
+        <v>1.6</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F42">
-        <v>2.8</v>
+        <v>0.8</v>
       </c>
       <c r="G42">
-        <v>3.972</v>
+        <v>1.433</v>
       </c>
       <c r="H42">
-        <v>-0.062</v>
+        <v>-0.06</v>
       </c>
       <c r="I42" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -1709,28 +1709,28 @@
         <v>11</v>
       </c>
       <c r="B43" s="2">
-        <v>45172</v>
+        <v>45156</v>
       </c>
       <c r="C43" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D43">
-        <v>0.8</v>
+        <v>1.267</v>
       </c>
       <c r="E43">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F43">
-        <v>-1.6</v>
+        <v>2.8</v>
       </c>
       <c r="G43">
-        <v>-2.111</v>
+        <v>3.972</v>
       </c>
       <c r="H43">
-        <v>-0.014</v>
+        <v>-0.062</v>
       </c>
       <c r="I43" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -1738,28 +1738,28 @@
         <v>11</v>
       </c>
       <c r="B44" s="2">
-        <v>45434</v>
+        <v>45172</v>
       </c>
       <c r="C44" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D44">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E44">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F44">
-        <v>0</v>
+        <v>-1.6</v>
       </c>
       <c r="G44">
-        <v>0.161</v>
+        <v>-2.111</v>
       </c>
       <c r="H44">
-        <v>-0.08500000000000001</v>
+        <v>-0.014</v>
       </c>
       <c r="I44" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -1767,28 +1767,28 @@
         <v>11</v>
       </c>
       <c r="B45" s="2">
-        <v>45440</v>
+        <v>45434</v>
       </c>
       <c r="C45" t="s">
         <v>13</v>
       </c>
       <c r="D45">
-        <v>1.067</v>
+        <v>1</v>
       </c>
       <c r="E45">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F45">
-        <v>2.2</v>
+        <v>0</v>
       </c>
       <c r="G45">
-        <v>2.939</v>
+        <v>0.161</v>
       </c>
       <c r="H45">
-        <v>-0.04</v>
+        <v>-0.08500000000000001</v>
       </c>
       <c r="I45" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -1796,25 +1796,25 @@
         <v>11</v>
       </c>
       <c r="B46" s="2">
-        <v>45443</v>
+        <v>45440</v>
       </c>
       <c r="C46" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D46">
-        <v>1.133</v>
+        <v>1.067</v>
       </c>
       <c r="E46">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F46">
-        <v>3.4</v>
+        <v>2.2</v>
       </c>
       <c r="G46">
-        <v>4.128</v>
+        <v>2.939</v>
       </c>
       <c r="H46">
-        <v>-0.09</v>
+        <v>-0.04</v>
       </c>
       <c r="I46" t="s">
         <v>35</v>
@@ -1825,28 +1825,28 @@
         <v>11</v>
       </c>
       <c r="B47" s="2">
-        <v>45453</v>
+        <v>45443</v>
       </c>
       <c r="C47" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D47">
-        <v>1.333</v>
+        <v>1.133</v>
       </c>
       <c r="E47">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F47">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="G47">
-        <v>0.239</v>
+        <v>4.128</v>
       </c>
       <c r="H47">
-        <v>-0.025</v>
+        <v>-0.09</v>
       </c>
       <c r="I47" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -1854,28 +1854,28 @@
         <v>11</v>
       </c>
       <c r="B48" s="2">
-        <v>45465</v>
+        <v>45453</v>
       </c>
       <c r="C48" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D48">
-        <v>1.4</v>
+        <v>1.333</v>
       </c>
       <c r="E48">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F48">
-        <v>-1.8</v>
+        <v>0</v>
       </c>
       <c r="G48">
-        <v>-2.367</v>
+        <v>0.239</v>
       </c>
       <c r="H48">
-        <v>0.022</v>
+        <v>-0.025</v>
       </c>
       <c r="I48" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -1883,28 +1883,28 @@
         <v>11</v>
       </c>
       <c r="B49" s="2">
-        <v>45466</v>
+        <v>45465</v>
       </c>
       <c r="C49" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D49">
-        <v>0.667</v>
+        <v>1.4</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F49">
-        <v>1</v>
+        <v>-1.8</v>
       </c>
       <c r="G49">
-        <v>1.383</v>
+        <v>-2.367</v>
       </c>
       <c r="H49">
-        <v>-0.011</v>
+        <v>0.022</v>
       </c>
       <c r="I49" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -1912,28 +1912,28 @@
         <v>11</v>
       </c>
       <c r="B50" s="2">
-        <v>45467</v>
+        <v>45466</v>
       </c>
       <c r="C50" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D50">
-        <v>0.533</v>
+        <v>0.667</v>
       </c>
       <c r="E50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F50">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="G50">
-        <v>2.033</v>
+        <v>1.383</v>
       </c>
       <c r="H50">
-        <v>-0.07000000000000001</v>
+        <v>-0.011</v>
       </c>
       <c r="I50" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -1941,28 +1941,28 @@
         <v>11</v>
       </c>
       <c r="B51" s="2">
-        <v>45475</v>
+        <v>45467</v>
       </c>
       <c r="C51" t="s">
         <v>12</v>
       </c>
       <c r="D51">
-        <v>0.2</v>
+        <v>0.533</v>
       </c>
       <c r="E51">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F51">
-        <v>-1.4</v>
+        <v>1.6</v>
       </c>
       <c r="G51">
-        <v>-1.517</v>
+        <v>2.033</v>
       </c>
       <c r="H51">
-        <v>0.024</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="I51" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -1970,28 +1970,28 @@
         <v>11</v>
       </c>
       <c r="B52" s="2">
-        <v>45480</v>
+        <v>45475</v>
       </c>
       <c r="C52" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="D52">
-        <v>0.667</v>
+        <v>0.2</v>
       </c>
       <c r="E52">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F52">
-        <v>2</v>
+        <v>-1.4</v>
       </c>
       <c r="G52">
-        <v>2.494</v>
+        <v>-1.517</v>
       </c>
       <c r="H52">
-        <v>-0.039</v>
+        <v>0.024</v>
       </c>
       <c r="I52" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -1999,28 +1999,28 @@
         <v>11</v>
       </c>
       <c r="B53" s="2">
-        <v>45487</v>
+        <v>45480</v>
       </c>
       <c r="C53" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D53">
-        <v>0.4</v>
+        <v>0.667</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F53">
-        <v>0.2</v>
+        <v>2</v>
       </c>
       <c r="G53">
-        <v>-0.017</v>
+        <v>2.494</v>
       </c>
       <c r="H53">
-        <v>0.008999999999999999</v>
+        <v>-0.039</v>
       </c>
       <c r="I53" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -2028,28 +2028,28 @@
         <v>11</v>
       </c>
       <c r="B54" s="2">
-        <v>45492</v>
+        <v>45487</v>
       </c>
       <c r="C54" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D54">
-        <v>0.667</v>
+        <v>0.4</v>
       </c>
       <c r="E54">
         <v>1</v>
       </c>
       <c r="F54">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="G54">
-        <v>1.35</v>
+        <v>-0.017</v>
       </c>
       <c r="H54">
-        <v>-0.018</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="I54" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -2057,28 +2057,28 @@
         <v>11</v>
       </c>
       <c r="B55" s="2">
-        <v>45496</v>
+        <v>45492</v>
       </c>
       <c r="C55" t="s">
         <v>16</v>
       </c>
       <c r="D55">
-        <v>0.467</v>
+        <v>0.667</v>
       </c>
       <c r="E55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F55">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="G55">
-        <v>1.783</v>
+        <v>1.35</v>
       </c>
       <c r="H55">
-        <v>-0.011</v>
+        <v>-0.018</v>
       </c>
       <c r="I55" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -2086,28 +2086,28 @@
         <v>11</v>
       </c>
       <c r="B56" s="2">
-        <v>45502</v>
+        <v>45496</v>
       </c>
       <c r="C56" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D56">
-        <v>0.533</v>
+        <v>0.467</v>
       </c>
       <c r="E56">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F56">
-        <v>-2.4</v>
+        <v>1.4</v>
       </c>
       <c r="G56">
-        <v>-3.428</v>
+        <v>1.783</v>
       </c>
       <c r="H56">
-        <v>0.054</v>
+        <v>-0.011</v>
       </c>
       <c r="I56" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -2115,28 +2115,28 @@
         <v>11</v>
       </c>
       <c r="B57" s="2">
-        <v>45514</v>
+        <v>45502</v>
       </c>
       <c r="C57" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D57">
-        <v>0.867</v>
+        <v>0.533</v>
       </c>
       <c r="E57">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F57">
-        <v>2.6</v>
+        <v>-2.4</v>
       </c>
       <c r="G57">
-        <v>3.278</v>
+        <v>-3.428</v>
       </c>
       <c r="H57">
-        <v>-0.07099999999999999</v>
+        <v>0.054</v>
       </c>
       <c r="I57" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -2144,28 +2144,28 @@
         <v>11</v>
       </c>
       <c r="B58" s="2">
-        <v>45535</v>
+        <v>45514</v>
       </c>
       <c r="C58" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D58">
-        <v>0.9330000000000001</v>
+        <v>0.867</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F58">
-        <v>0.8</v>
+        <v>2.6</v>
       </c>
       <c r="G58">
-        <v>1.011</v>
+        <v>3.278</v>
       </c>
       <c r="H58">
-        <v>-0.05</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="I58" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -2173,28 +2173,28 @@
         <v>11</v>
       </c>
       <c r="B59" s="2">
-        <v>45570</v>
+        <v>45535</v>
       </c>
       <c r="C59" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D59">
-        <v>0.4</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E59">
         <v>2</v>
       </c>
       <c r="F59">
-        <v>-0.8</v>
+        <v>0.8</v>
       </c>
       <c r="G59">
-        <v>-1.1</v>
+        <v>1.011</v>
       </c>
       <c r="H59">
-        <v>0.035</v>
+        <v>-0.05</v>
       </c>
       <c r="I59" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -2202,28 +2202,28 @@
         <v>11</v>
       </c>
       <c r="B60" s="2">
-        <v>45580</v>
+        <v>45570</v>
       </c>
       <c r="C60" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="D60">
-        <v>0.667</v>
+        <v>0.4</v>
       </c>
       <c r="E60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F60">
-        <v>1</v>
+        <v>-0.8</v>
       </c>
       <c r="G60">
-        <v>1.056</v>
+        <v>-1.1</v>
       </c>
       <c r="H60">
-        <v>-0.013</v>
+        <v>0.035</v>
       </c>
       <c r="I60" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -2231,28 +2231,28 @@
         <v>11</v>
       </c>
       <c r="B61" s="2">
-        <v>45649</v>
+        <v>45580</v>
       </c>
       <c r="C61" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D61">
-        <v>0.9330000000000001</v>
+        <v>0.667</v>
       </c>
       <c r="E61">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F61">
-        <v>-0.2</v>
+        <v>1</v>
       </c>
       <c r="G61">
-        <v>-0.289</v>
+        <v>1.056</v>
       </c>
       <c r="H61">
-        <v>-0.028</v>
+        <v>-0.013</v>
       </c>
       <c r="I61" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -2260,28 +2260,28 @@
         <v>11</v>
       </c>
       <c r="B62" s="2">
-        <v>45653</v>
+        <v>45649</v>
       </c>
       <c r="C62" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D62">
-        <v>0.4</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F62">
-        <v>-0.8</v>
+        <v>-0.2</v>
       </c>
       <c r="G62">
-        <v>-0.844</v>
+        <v>-0.289</v>
       </c>
       <c r="H62">
-        <v>-0.012</v>
+        <v>-0.028</v>
       </c>
       <c r="I62" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -2289,28 +2289,28 @@
         <v>11</v>
       </c>
       <c r="B63" s="2">
-        <v>45655</v>
+        <v>45653</v>
       </c>
       <c r="C63" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D63">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="E63">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F63">
-        <v>1.4</v>
+        <v>-0.8</v>
       </c>
       <c r="G63">
-        <v>1.989</v>
+        <v>-0.844</v>
       </c>
       <c r="H63">
-        <v>0.003</v>
+        <v>-0.012</v>
       </c>
       <c r="I63" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -2318,28 +2318,28 @@
         <v>11</v>
       </c>
       <c r="B64" s="2">
-        <v>45735</v>
+        <v>45655</v>
       </c>
       <c r="C64" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D64">
-        <v>0.333</v>
+        <v>0.8</v>
       </c>
       <c r="E64">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F64">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="G64">
-        <v>1.189</v>
+        <v>1.989</v>
       </c>
       <c r="H64">
-        <v>-0.051</v>
+        <v>0.003</v>
       </c>
       <c r="I64" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -2347,25 +2347,25 @@
         <v>11</v>
       </c>
       <c r="B65" s="2">
-        <v>45829</v>
+        <v>45735</v>
       </c>
       <c r="C65" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D65">
-        <v>0.267</v>
+        <v>0.333</v>
       </c>
       <c r="E65">
         <v>0</v>
       </c>
       <c r="F65">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="G65">
-        <v>0.911</v>
+        <v>1.189</v>
       </c>
       <c r="H65">
-        <v>-0.033</v>
+        <v>-0.051</v>
       </c>
       <c r="I65" t="s">
         <v>33</v>
@@ -2376,25 +2376,25 @@
         <v>11</v>
       </c>
       <c r="B66" s="2">
-        <v>45831</v>
+        <v>45829</v>
       </c>
       <c r="C66" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D66">
-        <v>0.4</v>
+        <v>0.267</v>
       </c>
       <c r="E66">
         <v>0</v>
       </c>
       <c r="F66">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="G66">
-        <v>1.483</v>
+        <v>0.911</v>
       </c>
       <c r="H66">
-        <v>-0.068</v>
+        <v>-0.033</v>
       </c>
       <c r="I66" t="s">
         <v>33</v>
@@ -2405,25 +2405,25 @@
         <v>11</v>
       </c>
       <c r="B67" s="2">
-        <v>45844</v>
+        <v>45831</v>
       </c>
       <c r="C67" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D67">
-        <v>0.467</v>
+        <v>0.4</v>
       </c>
       <c r="E67">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F67">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="G67">
-        <v>0.628</v>
+        <v>1.483</v>
       </c>
       <c r="H67">
-        <v>0.027</v>
+        <v>-0.068</v>
       </c>
       <c r="I67" t="s">
         <v>33</v>
@@ -2434,28 +2434,28 @@
         <v>11</v>
       </c>
       <c r="B68" s="2">
-        <v>45857</v>
+        <v>45844</v>
       </c>
       <c r="C68" t="s">
         <v>14</v>
       </c>
       <c r="D68">
-        <v>0.2</v>
+        <v>0.467</v>
       </c>
       <c r="E68">
         <v>1</v>
       </c>
       <c r="F68">
-        <v>-0.4</v>
+        <v>0.4</v>
       </c>
       <c r="G68">
-        <v>-0.433</v>
+        <v>0.628</v>
       </c>
       <c r="H68">
-        <v>0.002</v>
+        <v>0.027</v>
       </c>
       <c r="I68" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -2463,28 +2463,28 @@
         <v>11</v>
       </c>
       <c r="B69" s="2">
-        <v>45868</v>
+        <v>45857</v>
       </c>
       <c r="C69" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D69">
-        <v>0.667</v>
+        <v>0.2</v>
       </c>
       <c r="E69">
         <v>1</v>
       </c>
       <c r="F69">
-        <v>1</v>
+        <v>-0.4</v>
       </c>
       <c r="G69">
-        <v>1.439</v>
+        <v>-0.433</v>
       </c>
       <c r="H69">
-        <v>0.018</v>
+        <v>0.002</v>
       </c>
       <c r="I69" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -2492,28 +2492,28 @@
         <v>11</v>
       </c>
       <c r="B70" s="2">
-        <v>45886</v>
+        <v>45868</v>
       </c>
       <c r="C70" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D70">
-        <v>0.6</v>
+        <v>0.667</v>
       </c>
       <c r="E70">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F70">
-        <v>-0.2</v>
+        <v>1</v>
       </c>
       <c r="G70">
-        <v>-0.644</v>
+        <v>1.439</v>
       </c>
       <c r="H70">
-        <v>-0.005</v>
+        <v>0.018</v>
       </c>
       <c r="I70" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -2521,28 +2521,28 @@
         <v>11</v>
       </c>
       <c r="B71" s="2">
-        <v>45892</v>
+        <v>45886</v>
       </c>
       <c r="C71" t="s">
         <v>20</v>
       </c>
       <c r="D71">
-        <v>0.733</v>
+        <v>0.6</v>
       </c>
       <c r="E71">
         <v>2</v>
       </c>
       <c r="F71">
-        <v>0.2</v>
+        <v>-0.2</v>
       </c>
       <c r="G71">
-        <v>0.361</v>
+        <v>-0.644</v>
       </c>
       <c r="H71">
-        <v>-0.055</v>
+        <v>-0.005</v>
       </c>
       <c r="I71" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -2550,28 +2550,28 @@
         <v>11</v>
       </c>
       <c r="B72" s="2">
-        <v>45894</v>
+        <v>45892</v>
       </c>
       <c r="C72" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D72">
-        <v>1.2</v>
+        <v>0.733</v>
       </c>
       <c r="E72">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F72">
-        <v>-2.4</v>
+        <v>0.2</v>
       </c>
       <c r="G72">
-        <v>-2.606</v>
+        <v>0.361</v>
       </c>
       <c r="H72">
-        <v>0.068</v>
+        <v>-0.055</v>
       </c>
       <c r="I72" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -2579,25 +2579,25 @@
         <v>11</v>
       </c>
       <c r="B73" s="2">
-        <v>45897</v>
+        <v>45894</v>
       </c>
       <c r="C73" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D73">
-        <v>0.867</v>
+        <v>1.2</v>
       </c>
       <c r="E73">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F73">
-        <v>-1.4</v>
+        <v>-2.4</v>
       </c>
       <c r="G73">
-        <v>-1.789</v>
+        <v>-2.606</v>
       </c>
       <c r="H73">
-        <v>0.001</v>
+        <v>0.068</v>
       </c>
       <c r="I73" t="s">
         <v>34</v>
@@ -2608,25 +2608,25 @@
         <v>11</v>
       </c>
       <c r="B74" s="2">
-        <v>45941</v>
+        <v>45897</v>
       </c>
       <c r="C74" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D74">
-        <v>0.9330000000000001</v>
+        <v>0.867</v>
       </c>
       <c r="E74">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F74">
-        <v>-2.2</v>
+        <v>-1.4</v>
       </c>
       <c r="G74">
-        <v>-2.9</v>
+        <v>-1.789</v>
       </c>
       <c r="H74">
-        <v>-0.001</v>
+        <v>0.001</v>
       </c>
       <c r="I74" t="s">
         <v>34</v>
@@ -2637,25 +2637,25 @@
         <v>11</v>
       </c>
       <c r="B75" s="2">
-        <v>46160</v>
+        <v>45941</v>
       </c>
       <c r="C75" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D75">
-        <v>0.467</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E75">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F75">
-        <v>-1.6</v>
+        <v>-2.2</v>
       </c>
       <c r="G75">
-        <v>-1.972</v>
+        <v>-2.9</v>
       </c>
       <c r="H75">
-        <v>0.029</v>
+        <v>-0.001</v>
       </c>
       <c r="I75" t="s">
         <v>34</v>
@@ -2666,28 +2666,28 @@
         <v>11</v>
       </c>
       <c r="B76" s="2">
-        <v>46164</v>
+        <v>46160</v>
       </c>
       <c r="C76" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D76">
-        <v>1</v>
+        <v>0.467</v>
       </c>
       <c r="E76">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F76">
-        <v>1</v>
+        <v>-1.6</v>
       </c>
       <c r="G76">
-        <v>1.417</v>
+        <v>-1.972</v>
       </c>
       <c r="H76">
-        <v>0.011</v>
+        <v>0.029</v>
       </c>
       <c r="I76" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -2695,28 +2695,28 @@
         <v>11</v>
       </c>
       <c r="B77" s="2">
-        <v>46173</v>
+        <v>46164</v>
       </c>
       <c r="C77" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D77">
-        <v>0.733</v>
+        <v>1</v>
       </c>
       <c r="E77">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F77">
-        <v>-0.8</v>
+        <v>1</v>
       </c>
       <c r="G77">
-        <v>-1.167</v>
+        <v>1.417</v>
       </c>
       <c r="H77">
-        <v>0.023</v>
+        <v>0.011</v>
       </c>
       <c r="I77" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -2724,25 +2724,25 @@
         <v>11</v>
       </c>
       <c r="B78" s="2">
-        <v>46201</v>
+        <v>46173</v>
       </c>
       <c r="C78" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D78">
-        <v>1.067</v>
+        <v>0.733</v>
       </c>
       <c r="E78">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F78">
-        <v>-2.8</v>
+        <v>-0.8</v>
       </c>
       <c r="G78">
-        <v>-3.983</v>
+        <v>-1.167</v>
       </c>
       <c r="H78">
-        <v>0.002</v>
+        <v>0.023</v>
       </c>
       <c r="I78" t="s">
         <v>34</v>
@@ -2753,25 +2753,25 @@
         <v>11</v>
       </c>
       <c r="B79" s="2">
-        <v>46212</v>
+        <v>46201</v>
       </c>
       <c r="C79" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D79">
-        <v>0.4</v>
+        <v>1.067</v>
       </c>
       <c r="E79">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F79">
-        <v>-1.8</v>
+        <v>-2.8</v>
       </c>
       <c r="G79">
-        <v>-2.756</v>
+        <v>-3.983</v>
       </c>
       <c r="H79">
-        <v>0.015</v>
+        <v>0.002</v>
       </c>
       <c r="I79" t="s">
         <v>34</v>
@@ -2782,28 +2782,28 @@
         <v>11</v>
       </c>
       <c r="B80" s="2">
-        <v>46221</v>
+        <v>46212</v>
       </c>
       <c r="C80" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D80">
-        <v>0.867</v>
+        <v>0.4</v>
       </c>
       <c r="E80">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F80">
-        <v>1.6</v>
+        <v>-1.8</v>
       </c>
       <c r="G80">
-        <v>1.85</v>
+        <v>-2.756</v>
       </c>
       <c r="H80">
-        <v>-0.027</v>
+        <v>0.015</v>
       </c>
       <c r="I80" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -2811,10 +2811,10 @@
         <v>11</v>
       </c>
       <c r="B81" s="2">
-        <v>46222</v>
+        <v>46221</v>
       </c>
       <c r="C81" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D81">
         <v>0.867</v>
@@ -2826,7 +2826,7 @@
         <v>1.6</v>
       </c>
       <c r="G81">
-        <v>1.861</v>
+        <v>1.85</v>
       </c>
       <c r="H81">
         <v>-0.027</v>
@@ -2840,27 +2840,85 @@
         <v>11</v>
       </c>
       <c r="B82" s="2">
+        <v>46222</v>
+      </c>
+      <c r="C82" t="s">
+        <v>22</v>
+      </c>
+      <c r="D82">
+        <v>0.867</v>
+      </c>
+      <c r="E82">
+        <v>1</v>
+      </c>
+      <c r="F82">
+        <v>1.6</v>
+      </c>
+      <c r="G82">
+        <v>1.861</v>
+      </c>
+      <c r="H82">
+        <v>-0.027</v>
+      </c>
+      <c r="I82" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9">
+      <c r="A83" t="s">
+        <v>11</v>
+      </c>
+      <c r="B83" s="2">
         <v>46243</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C83" t="s">
         <v>23</v>
       </c>
-      <c r="D82">
+      <c r="D83">
         <v>0.333</v>
       </c>
-      <c r="E82">
+      <c r="E83">
         <v>0</v>
       </c>
-      <c r="F82">
-        <v>1</v>
-      </c>
-      <c r="G82">
+      <c r="F83">
+        <v>1</v>
+      </c>
+      <c r="G83">
         <v>1.089</v>
       </c>
-      <c r="H82">
+      <c r="H83">
         <v>0.001</v>
       </c>
-      <c r="I82" t="s">
+      <c r="I83" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9">
+      <c r="A84" t="s">
+        <v>11</v>
+      </c>
+      <c r="B84" s="2">
+        <v>46249</v>
+      </c>
+      <c r="C84" t="s">
+        <v>12</v>
+      </c>
+      <c r="D84">
+        <v>0.667</v>
+      </c>
+      <c r="E84">
+        <v>1</v>
+      </c>
+      <c r="F84">
+        <v>1</v>
+      </c>
+      <c r="G84">
+        <v>1.439</v>
+      </c>
+      <c r="H84">
+        <v>-0.096</v>
+      </c>
+      <c r="I84" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>